<commit_message>
Run unit tests on screening modules, correct mortality after screening, check IMABC internal validation
</commit_message>
<xml_diff>
--- a/tests/test_screening_data.xlsx
+++ b/tests/test_screening_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36286245-274D-0242-AB42-31C63E7E86FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{001C2D92-8BB8-CE4D-B666-3A508F4722F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10580" yWindow="760" windowWidth="19660" windowHeight="17400" xr2:uid="{C01DA78E-62CC-6E49-850F-A2DB27289041}"/>
+    <workbookView xWindow="15120" yWindow="760" windowWidth="15120" windowHeight="17780" xr2:uid="{C01DA78E-62CC-6E49-850F-A2DB27289041}"/>
   </bookViews>
   <sheets>
     <sheet name="m_patient" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="57">
   <si>
     <t>pt_id</t>
   </si>
@@ -205,6 +205,9 @@
   </si>
   <si>
     <t>ct_2_nosurv_b_L</t>
+  </si>
+  <si>
+    <t>lesion_id</t>
   </si>
 </sst>
 </file>
@@ -886,46 +889,28 @@
       <c r="V3">
         <v>0</v>
       </c>
-      <c r="W3">
-        <v>0</v>
-      </c>
       <c r="X3">
         <v>0</v>
       </c>
       <c r="Y3">
         <v>0</v>
       </c>
-      <c r="Z3">
-        <v>0</v>
-      </c>
       <c r="AA3">
         <v>0</v>
       </c>
-      <c r="AB3">
-        <v>0</v>
-      </c>
       <c r="AC3">
         <v>0</v>
       </c>
       <c r="AD3">
         <v>0</v>
       </c>
-      <c r="AE3">
-        <v>0</v>
-      </c>
       <c r="AF3">
         <v>0</v>
       </c>
-      <c r="AG3">
-        <v>0</v>
-      </c>
       <c r="AH3">
         <v>0</v>
       </c>
       <c r="AI3">
-        <v>0</v>
-      </c>
-      <c r="AJ3">
         <v>0</v>
       </c>
     </row>
@@ -1006,47 +991,29 @@
       <c r="V4">
         <v>1</v>
       </c>
-      <c r="W4">
-        <v>0</v>
-      </c>
       <c r="X4">
         <v>1</v>
       </c>
       <c r="Y4">
         <v>1</v>
       </c>
-      <c r="Z4">
-        <v>0</v>
-      </c>
       <c r="AA4">
         <v>1</v>
       </c>
-      <c r="AB4">
-        <v>0</v>
-      </c>
       <c r="AC4">
         <v>1</v>
       </c>
       <c r="AD4">
         <v>1</v>
       </c>
-      <c r="AE4">
-        <v>0</v>
-      </c>
       <c r="AF4">
         <v>1</v>
       </c>
-      <c r="AG4">
-        <v>0</v>
-      </c>
       <c r="AH4">
         <v>1</v>
       </c>
       <c r="AI4">
         <v>1</v>
-      </c>
-      <c r="AJ4">
-        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:36" x14ac:dyDescent="0.2">
@@ -1126,33 +1093,21 @@
       <c r="V5">
         <v>2</v>
       </c>
-      <c r="W5">
-        <v>0</v>
-      </c>
       <c r="X5">
         <v>2</v>
       </c>
       <c r="Y5">
         <v>1</v>
       </c>
-      <c r="Z5">
-        <v>0</v>
-      </c>
       <c r="AA5">
         <v>3</v>
       </c>
-      <c r="AB5">
-        <v>0</v>
-      </c>
       <c r="AC5">
         <v>3</v>
       </c>
       <c r="AD5">
         <v>2</v>
       </c>
-      <c r="AE5">
-        <v>0</v>
-      </c>
       <c r="AF5">
         <v>3</v>
       </c>
@@ -1164,9 +1119,6 @@
       </c>
       <c r="AI5">
         <v>3</v>
-      </c>
-      <c r="AJ5">
-        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:36" x14ac:dyDescent="0.2">
@@ -1276,17 +1228,11 @@
       <c r="AF6">
         <v>2</v>
       </c>
-      <c r="AG6">
-        <v>0</v>
-      </c>
       <c r="AH6">
         <v>1</v>
       </c>
       <c r="AI6">
         <v>2</v>
-      </c>
-      <c r="AJ6">
-        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.2">
@@ -1381,32 +1327,20 @@
       <c r="AA7">
         <v>3</v>
       </c>
-      <c r="AB7">
-        <v>0</v>
-      </c>
       <c r="AC7">
         <v>4</v>
       </c>
       <c r="AD7">
         <v>1</v>
       </c>
-      <c r="AE7">
-        <v>0</v>
-      </c>
       <c r="AF7">
         <v>3</v>
-      </c>
-      <c r="AG7">
-        <v>0</v>
       </c>
       <c r="AH7">
         <v>4</v>
       </c>
       <c r="AI7">
         <v>1</v>
-      </c>
-      <c r="AJ7">
-        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:36" x14ac:dyDescent="0.2">
@@ -1486,23 +1420,14 @@
       <c r="V8">
         <v>2</v>
       </c>
-      <c r="W8">
-        <v>0</v>
-      </c>
       <c r="X8">
         <v>4</v>
       </c>
       <c r="Y8">
         <v>0</v>
       </c>
-      <c r="Z8">
-        <v>0</v>
-      </c>
       <c r="AA8">
         <v>2</v>
-      </c>
-      <c r="AB8">
-        <v>0</v>
       </c>
       <c r="AC8">
         <v>4</v>
@@ -1510,23 +1435,14 @@
       <c r="AD8">
         <v>1</v>
       </c>
-      <c r="AE8">
-        <v>0</v>
-      </c>
       <c r="AF8">
         <v>2</v>
-      </c>
-      <c r="AG8">
-        <v>0</v>
       </c>
       <c r="AH8">
         <v>4</v>
       </c>
       <c r="AI8">
         <v>1</v>
-      </c>
-      <c r="AJ8">
-        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:36" x14ac:dyDescent="0.2">
@@ -1606,23 +1522,14 @@
       <c r="V9">
         <v>3</v>
       </c>
-      <c r="W9">
-        <v>0</v>
-      </c>
       <c r="X9">
         <v>5</v>
       </c>
       <c r="Y9">
         <v>1</v>
       </c>
-      <c r="Z9">
-        <v>0</v>
-      </c>
       <c r="AA9">
         <v>3</v>
-      </c>
-      <c r="AB9">
-        <v>0</v>
       </c>
       <c r="AC9">
         <v>4</v>
@@ -1636,17 +1543,11 @@
       <c r="AF9">
         <v>3</v>
       </c>
-      <c r="AG9">
-        <v>0</v>
-      </c>
       <c r="AH9">
         <v>4</v>
       </c>
       <c r="AI9">
         <v>2</v>
-      </c>
-      <c r="AJ9">
-        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:36" x14ac:dyDescent="0.2">
@@ -1726,23 +1627,14 @@
       <c r="V10">
         <v>3</v>
       </c>
-      <c r="W10">
-        <v>0</v>
-      </c>
       <c r="X10">
         <v>5</v>
       </c>
       <c r="Y10">
         <v>0</v>
       </c>
-      <c r="Z10">
-        <v>0</v>
-      </c>
       <c r="AA10">
         <v>3</v>
-      </c>
-      <c r="AB10">
-        <v>0</v>
       </c>
       <c r="AC10">
         <v>5</v>
@@ -1750,22 +1642,13 @@
       <c r="AD10">
         <v>0</v>
       </c>
-      <c r="AE10">
-        <v>0</v>
-      </c>
       <c r="AF10">
         <v>3</v>
-      </c>
-      <c r="AG10">
-        <v>0</v>
       </c>
       <c r="AH10">
         <v>5</v>
       </c>
       <c r="AI10">
-        <v>0</v>
-      </c>
-      <c r="AJ10">
         <v>0</v>
       </c>
     </row>
@@ -1776,241 +1659,273 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFC853AB-1B40-724B-B920-12502C063EDC}">
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>56</v>
       </c>
       <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" t="s">
-        <v>2</v>
-      </c>
       <c r="F1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>27</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>42</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>43</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>44</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
+        <f t="shared" ref="B2:B4" si="0">IF(A2&lt;&gt;A1, 1, B1+1)</f>
+        <v>1</v>
+      </c>
+      <c r="C2">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A2,m_patient!$A:$A,0))</f>
         <v>3</v>
       </c>
-      <c r="C2">
-        <v>3</v>
-      </c>
       <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2">
         <v>10</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A2,m_patient!$A:$A,0))</f>
         <v>10</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A2,m_patient!$A:$A,0))</f>
         <v>90</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C3">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A3,m_patient!$A:$A,0))</f>
         <v>3</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>61</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>70</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A3,m_patient!$A:$A,0))</f>
         <v>10</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A3,m_patient!$A:$A,0))</f>
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C4">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A4,m_patient!$A:$A,0))</f>
         <v>3</v>
       </c>
-      <c r="C4">
-        <v>3</v>
-      </c>
       <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4">
         <v>10</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A4,m_patient!$A:$A,0))</f>
         <v>10</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A4,m_patient!$A:$A,0))</f>
         <v>20</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2</v>
       </c>
       <c r="B5">
+        <f>IF(A5&lt;&gt;A4, 1, B4+1)</f>
+        <v>2</v>
+      </c>
+      <c r="C5">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A5,m_patient!$A:$A,0))</f>
         <v>3</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <v>61</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>70</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A5,m_patient!$A:$A,0))</f>
         <v>10</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A5,m_patient!$A:$A,0))</f>
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>3</v>
       </c>
       <c r="B6">
+        <f t="shared" ref="B6:B23" si="1">IF(A6&lt;&gt;A5, 1, B5+1)</f>
+        <v>1</v>
+      </c>
+      <c r="C6">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A6,m_patient!$A:$A,0))</f>
         <v>3</v>
       </c>
-      <c r="C6">
-        <v>3</v>
-      </c>
       <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="E6">
         <v>10</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A6,m_patient!$A:$A,0))</f>
         <v>10</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A6,m_patient!$A:$A,0))</f>
         <v>90</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>3</v>
       </c>
       <c r="B7">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="C7">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A7,m_patient!$A:$A,0))</f>
         <v>3</v>
       </c>
-      <c r="C7">
+      <c r="D7">
         <v>61</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>70</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A7,m_patient!$A:$A,0))</f>
         <v>10</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A7,m_patient!$A:$A,0))</f>
         <v>90</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>3</v>
       </c>
       <c r="B8">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="C8">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A8,m_patient!$A:$A,0))</f>
         <v>3</v>
       </c>
-      <c r="C8">
+      <c r="D8">
         <v>40</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>52</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A8,m_patient!$A:$A,0))</f>
         <v>10</v>
       </c>
-      <c r="F8">
+      <c r="G8">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A8,m_patient!$A:$A,0))</f>
         <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>4</v>
       </c>
       <c r="B9">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="C9">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A9,m_patient!$A:$A,0))</f>
         <v>46</v>
       </c>
-      <c r="C9">
+      <c r="D9">
         <v>46</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>52</v>
       </c>
-      <c r="E9">
+      <c r="F9">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A9,m_patient!$A:$A,0))</f>
         <v>52</v>
       </c>
-      <c r="F9">
+      <c r="G9">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A9,m_patient!$A:$A,0))</f>
         <v>100</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>38</v>
-      </c>
-      <c r="H9">
-        <v>50</v>
       </c>
       <c r="I9">
         <v>50</v>
@@ -2021,32 +1936,36 @@
       <c r="K9">
         <v>50</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L9">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>4</v>
       </c>
       <c r="B10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="C10">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A10,m_patient!$A:$A,0))</f>
         <v>46</v>
       </c>
-      <c r="C10">
+      <c r="D10">
         <v>47</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>60</v>
       </c>
-      <c r="E10">
+      <c r="F10">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A10,m_patient!$A:$A,0))</f>
         <v>52</v>
       </c>
-      <c r="F10">
+      <c r="G10">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A10,m_patient!$A:$A,0))</f>
         <v>100</v>
       </c>
-      <c r="H10">
-        <v>50</v>
-      </c>
       <c r="I10">
         <v>50</v>
       </c>
@@ -2056,32 +1975,36 @@
       <c r="K10">
         <v>50</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L10">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>4</v>
       </c>
       <c r="B11">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="C11">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A11,m_patient!$A:$A,0))</f>
         <v>46</v>
       </c>
-      <c r="C11">
+      <c r="D11">
         <v>48</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>60</v>
       </c>
-      <c r="E11">
+      <c r="F11">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A11,m_patient!$A:$A,0))</f>
         <v>52</v>
       </c>
-      <c r="F11">
+      <c r="G11">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A11,m_patient!$A:$A,0))</f>
         <v>100</v>
       </c>
-      <c r="H11">
-        <v>50</v>
-      </c>
       <c r="I11">
         <v>50</v>
       </c>
@@ -2091,66 +2014,74 @@
       <c r="K11">
         <v>50</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L11">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>4</v>
       </c>
       <c r="B12">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="C12">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A12,m_patient!$A:$A,0))</f>
         <v>46</v>
       </c>
-      <c r="C12">
+      <c r="D12">
         <v>65</v>
       </c>
-      <c r="D12">
+      <c r="E12">
         <v>72</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A12,m_patient!$A:$A,0))</f>
         <v>52</v>
       </c>
-      <c r="F12">
+      <c r="G12">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A12,m_patient!$A:$A,0))</f>
         <v>100</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <v>70</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>65</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>5</v>
       </c>
       <c r="B13">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="C13">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A13,m_patient!$A:$A,0))</f>
         <v>46</v>
       </c>
-      <c r="C13">
+      <c r="D13">
         <v>46</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <v>62</v>
       </c>
-      <c r="E13">
+      <c r="F13">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A13,m_patient!$A:$A,0))</f>
         <v>56</v>
       </c>
-      <c r="F13">
+      <c r="G13">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A13,m_patient!$A:$A,0))</f>
         <v>70</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>37</v>
-      </c>
-      <c r="H13">
-        <v>50</v>
       </c>
       <c r="I13">
         <v>50</v>
@@ -2161,280 +2092,323 @@
       <c r="K13">
         <v>50</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L13">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>5</v>
       </c>
       <c r="B14">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="C14">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A14,m_patient!$A:$A,0))</f>
         <v>46</v>
       </c>
-      <c r="C14">
+      <c r="D14">
         <v>51</v>
       </c>
-      <c r="D14">
+      <c r="E14">
         <v>56</v>
       </c>
-      <c r="E14">
+      <c r="F14">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A14,m_patient!$A:$A,0))</f>
         <v>56</v>
       </c>
-      <c r="F14">
+      <c r="G14">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A14,m_patient!$A:$A,0))</f>
         <v>70</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>5</v>
       </c>
       <c r="B15">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="C15">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A15,m_patient!$A:$A,0))</f>
         <v>46</v>
       </c>
-      <c r="C15">
+      <c r="D15">
         <v>56</v>
       </c>
-      <c r="D15">
+      <c r="E15">
         <v>59</v>
       </c>
-      <c r="E15">
+      <c r="F15">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A15,m_patient!$A:$A,0))</f>
         <v>56</v>
       </c>
-      <c r="F15">
+      <c r="G15">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A15,m_patient!$A:$A,0))</f>
         <v>70</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>6</v>
       </c>
       <c r="B16">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="C16">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A16,m_patient!$A:$A,0))</f>
         <v>63</v>
       </c>
-      <c r="C16">
+      <c r="D16">
         <v>63</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <v>82</v>
       </c>
-      <c r="E16">
+      <c r="F16">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A16,m_patient!$A:$A,0))</f>
         <v>82</v>
       </c>
-      <c r="F16">
+      <c r="G16">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A16,m_patient!$A:$A,0))</f>
         <v>95</v>
       </c>
-      <c r="H16">
+      <c r="I16">
         <v>70</v>
       </c>
-      <c r="I16">
+      <c r="J16">
         <v>65</v>
       </c>
-      <c r="J16">
+      <c r="K16">
         <v>70</v>
       </c>
-      <c r="K16">
+      <c r="L16">
         <v>65</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>7</v>
       </c>
       <c r="B17">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="C17">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A17,m_patient!$A:$A,0))</f>
         <v>63</v>
       </c>
-      <c r="C17">
+      <c r="D17">
         <v>63</v>
       </c>
-      <c r="D17">
+      <c r="E17">
         <v>71</v>
       </c>
-      <c r="E17">
+      <c r="F17">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A17,m_patient!$A:$A,0))</f>
         <v>71</v>
       </c>
-      <c r="F17">
+      <c r="G17">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A17,m_patient!$A:$A,0))</f>
         <v>66</v>
       </c>
-      <c r="I17">
+      <c r="J17">
         <v>65</v>
       </c>
-      <c r="K17">
+      <c r="L17">
         <v>65</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>8</v>
       </c>
       <c r="B18">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="C18">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A18,m_patient!$A:$A,0))</f>
         <v>63</v>
       </c>
-      <c r="C18">
+      <c r="D18">
         <v>63</v>
       </c>
-      <c r="D18">
+      <c r="E18">
         <v>67</v>
       </c>
-      <c r="E18">
+      <c r="F18">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A18,m_patient!$A:$A,0))</f>
         <v>67</v>
       </c>
-      <c r="F18">
+      <c r="G18">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A18,m_patient!$A:$A,0))</f>
         <v>100</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>39</v>
       </c>
-      <c r="I18">
+      <c r="J18">
         <v>65</v>
       </c>
-      <c r="K18">
+      <c r="L18">
         <v>65</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>8</v>
       </c>
       <c r="B19">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="C19">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A19,m_patient!$A:$A,0))</f>
         <v>63</v>
       </c>
-      <c r="C19">
+      <c r="D19">
         <v>63</v>
       </c>
-      <c r="D19">
+      <c r="E19">
         <v>67</v>
       </c>
-      <c r="E19">
+      <c r="F19">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A19,m_patient!$A:$A,0))</f>
         <v>67</v>
       </c>
-      <c r="F19">
+      <c r="G19">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A19,m_patient!$A:$A,0))</f>
         <v>100</v>
       </c>
-      <c r="I19">
+      <c r="J19">
         <v>65</v>
       </c>
-      <c r="K19">
+      <c r="L19">
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>8</v>
       </c>
       <c r="B20">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="C20">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A20,m_patient!$A:$A,0))</f>
         <v>63</v>
       </c>
-      <c r="C20">
+      <c r="D20">
         <v>63</v>
       </c>
-      <c r="D20">
+      <c r="E20">
         <v>67</v>
       </c>
-      <c r="E20">
+      <c r="F20">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A20,m_patient!$A:$A,0))</f>
         <v>67</v>
       </c>
-      <c r="F20">
+      <c r="G20">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A20,m_patient!$A:$A,0))</f>
         <v>100</v>
       </c>
-      <c r="I20">
+      <c r="J20">
         <v>65</v>
       </c>
-      <c r="K20">
+      <c r="L20">
         <v>65</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>8</v>
       </c>
       <c r="B21">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="C21">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A21,m_patient!$A:$A,0))</f>
         <v>63</v>
       </c>
-      <c r="C21">
+      <c r="D21">
         <v>64</v>
       </c>
-      <c r="D21">
+      <c r="E21">
         <v>80</v>
       </c>
-      <c r="E21">
+      <c r="F21">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A21,m_patient!$A:$A,0))</f>
         <v>67</v>
       </c>
-      <c r="F21">
+      <c r="G21">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A21,m_patient!$A:$A,0))</f>
         <v>100</v>
       </c>
-      <c r="I21">
+      <c r="J21">
         <v>65</v>
       </c>
-      <c r="K21">
+      <c r="L21">
         <v>65</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>8</v>
       </c>
       <c r="B22">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="C22">
         <v>63</v>
       </c>
-      <c r="C22">
+      <c r="D22">
         <v>67</v>
       </c>
-      <c r="D22">
+      <c r="E22">
         <v>80</v>
       </c>
-      <c r="E22">
+      <c r="F22">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A22,m_patient!$A:$A,0))</f>
         <v>67</v>
       </c>
-      <c r="F22">
+      <c r="G22">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A22,m_patient!$A:$A,0))</f>
         <v>100</v>
       </c>
-      <c r="K22">
+      <c r="L22">
         <v>68</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>9</v>
       </c>
       <c r="B23">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="C23">
         <f>INDEX(m_patient!B:B,MATCH(m_lesion!$A23,m_patient!$A:$A,0))</f>
         <v>110</v>
       </c>
-      <c r="C23">
+      <c r="D23">
         <v>110</v>
       </c>
-      <c r="D23">
+      <c r="E23">
         <v>111</v>
       </c>
-      <c r="E23">
+      <c r="F23">
         <f>INDEX(m_patient!C:C,MATCH(m_lesion!$A23,m_patient!$A:$A,0))</f>
         <v>111</v>
       </c>
-      <c r="F23">
+      <c r="G23">
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A23,m_patient!$A:$A,0))</f>
         <v>80</v>
       </c>

</xml_diff>

<commit_message>
Update tests and code for healthy and preclinical screening
</commit_message>
<xml_diff>
--- a/tests/test_screening_data.xlsx
+++ b/tests/test_screening_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{001C2D92-8BB8-CE4D-B666-3A508F4722F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85CEEFDA-E9C5-C84D-9121-81193C7A5F92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15120" yWindow="760" windowWidth="15120" windowHeight="17780" xr2:uid="{C01DA78E-62CC-6E49-850F-A2DB27289041}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" activeTab="1" xr2:uid="{C01DA78E-62CC-6E49-850F-A2DB27289041}"/>
   </bookViews>
   <sheets>
     <sheet name="m_patient" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="50">
   <si>
     <t>pt_id</t>
   </si>
@@ -60,24 +60,6 @@
     <t>time_H_Pj</t>
   </si>
   <si>
-    <t>ct_1_c_HL</t>
-  </si>
-  <si>
-    <t>ct_2_s_HL</t>
-  </si>
-  <si>
-    <t>ct_1_c_HP</t>
-  </si>
-  <si>
-    <t>ct_2_s_HP</t>
-  </si>
-  <si>
-    <t>ct_1_c_P</t>
-  </si>
-  <si>
-    <t>ct_2_s_P</t>
-  </si>
-  <si>
     <t>ct_1_b_P</t>
   </si>
   <si>
@@ -114,12 +96,6 @@
     <t>time_H_Dc</t>
   </si>
   <si>
-    <t>ct_2_c_P</t>
-  </si>
-  <si>
-    <t>ct_2_b_P</t>
-  </si>
-  <si>
     <t>purpose</t>
   </si>
   <si>
@@ -165,9 +141,6 @@
     <t>preclinical detection</t>
   </si>
   <si>
-    <t>test_1_nosurv_time_detected</t>
-  </si>
-  <si>
     <t>test_2_nosurv_time_detected</t>
   </si>
   <si>
@@ -177,37 +150,43 @@
     <t>test_2_surv_time_detected</t>
   </si>
   <si>
-    <t>ct_1_surv_c_L</t>
-  </si>
-  <si>
-    <t>ct_1_surv_b_L</t>
-  </si>
-  <si>
-    <t>ct_2_surv_s_L</t>
-  </si>
-  <si>
-    <t>ct_2_surv_c_L</t>
-  </si>
-  <si>
-    <t>ct_2_surv_b_L</t>
-  </si>
-  <si>
-    <t>ct_1_nosurv_c_L</t>
-  </si>
-  <si>
-    <t>ct_1_nosurv_b_L</t>
-  </si>
-  <si>
-    <t>ct_2_nosurv_s_L</t>
-  </si>
-  <si>
-    <t>ct_2_nosurv_c_L</t>
-  </si>
-  <si>
-    <t>ct_2_nosurv_b_L</t>
-  </si>
-  <si>
     <t>lesion_id</t>
+  </si>
+  <si>
+    <t>ct_10_HL</t>
+  </si>
+  <si>
+    <t>ct_1_HL</t>
+  </si>
+  <si>
+    <t>ct_10_HP</t>
+  </si>
+  <si>
+    <t>ct_1_HP</t>
+  </si>
+  <si>
+    <t>ct_10_s_P</t>
+  </si>
+  <si>
+    <t>ct_10_b_P</t>
+  </si>
+  <si>
+    <t>ct_1_s_P</t>
+  </si>
+  <si>
+    <t>ct_1_s_L</t>
+  </si>
+  <si>
+    <t>ct_1_b_L</t>
+  </si>
+  <si>
+    <t>ct_10_s_L</t>
+  </si>
+  <si>
+    <t>ct_10_b_L</t>
+  </si>
+  <si>
+    <t>test_10_time_detected</t>
   </si>
 </sst>
 </file>
@@ -579,10 +558,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE386AE5-7C58-FF46-B22F-83A12B65CF2D}">
-  <dimension ref="A1:AJ10"/>
+  <dimension ref="A1:AC10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -593,106 +572,85 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" t="s">
         <v>14</v>
       </c>
-      <c r="E1" t="s">
+      <c r="K1" t="s">
         <v>15</v>
       </c>
-      <c r="F1" t="s">
+      <c r="L1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M1" t="s">
+        <v>17</v>
+      </c>
+      <c r="N1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O1" t="s">
         <v>16</v>
-      </c>
-      <c r="G1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H1" t="s">
-        <v>18</v>
-      </c>
-      <c r="I1" t="s">
-        <v>19</v>
-      </c>
-      <c r="J1" t="s">
-        <v>20</v>
-      </c>
-      <c r="K1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M1" t="s">
-        <v>23</v>
-      </c>
-      <c r="N1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O1" t="s">
-        <v>22</v>
       </c>
       <c r="P1" t="s">
         <v>4</v>
       </c>
       <c r="Q1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="R1" t="s">
+        <v>38</v>
+      </c>
+      <c r="S1" t="s">
+        <v>39</v>
+      </c>
+      <c r="T1" t="s">
+        <v>40</v>
+      </c>
+      <c r="U1" t="s">
+        <v>41</v>
+      </c>
+      <c r="V1" t="s">
+        <v>42</v>
+      </c>
+      <c r="W1" t="s">
+        <v>43</v>
+      </c>
+      <c r="X1" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y1" t="s">
         <v>7</v>
       </c>
-      <c r="S1" t="s">
-        <v>8</v>
-      </c>
-      <c r="T1" t="s">
-        <v>9</v>
-      </c>
-      <c r="U1" t="s">
-        <v>10</v>
-      </c>
-      <c r="V1" t="s">
-        <v>11</v>
-      </c>
-      <c r="W1" t="s">
-        <v>13</v>
-      </c>
-      <c r="X1" t="s">
-        <v>12</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>25</v>
-      </c>
       <c r="Z1" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="AA1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="AB1" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="AC1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>55</v>
-      </c>
-      <c r="AF1" t="s">
         <v>46</v>
       </c>
-      <c r="AG1" t="s">
-        <v>47</v>
-      </c>
-      <c r="AH1" t="s">
-        <v>48</v>
-      </c>
-      <c r="AI1" t="s">
-        <v>49</v>
-      </c>
-      <c r="AJ1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -752,7 +710,7 @@
         <v>70</v>
       </c>
       <c r="Q2" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="R2">
         <v>0</v>
@@ -776,43 +734,19 @@
         <v>0</v>
       </c>
       <c r="Y2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB2">
-        <v>1</v>
-      </c>
-      <c r="AC2">
-        <v>0</v>
-      </c>
-      <c r="AD2">
-        <v>0</v>
-      </c>
-      <c r="AE2">
-        <v>1</v>
-      </c>
-      <c r="AF2">
-        <v>0</v>
-      </c>
-      <c r="AG2">
-        <v>1</v>
-      </c>
-      <c r="AH2">
-        <v>0</v>
-      </c>
-      <c r="AI2">
-        <v>0</v>
-      </c>
-      <c r="AJ2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -872,7 +806,7 @@
         <v>20</v>
       </c>
       <c r="Q3" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="R3">
         <v>0</v>
@@ -892,29 +826,14 @@
       <c r="X3">
         <v>0</v>
       </c>
-      <c r="Y3">
-        <v>0</v>
-      </c>
-      <c r="AA3">
-        <v>0</v>
-      </c>
-      <c r="AC3">
-        <v>0</v>
-      </c>
-      <c r="AD3">
-        <v>0</v>
-      </c>
-      <c r="AF3">
-        <v>0</v>
-      </c>
-      <c r="AH3">
-        <v>0</v>
-      </c>
-      <c r="AI3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="Z3">
+        <v>0</v>
+      </c>
+      <c r="AB3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -974,7 +893,7 @@
         <v>70</v>
       </c>
       <c r="Q4" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="R4">
         <v>0</v>
@@ -994,29 +913,14 @@
       <c r="X4">
         <v>1</v>
       </c>
-      <c r="Y4">
-        <v>1</v>
-      </c>
-      <c r="AA4">
-        <v>1</v>
-      </c>
-      <c r="AC4">
-        <v>1</v>
-      </c>
-      <c r="AD4">
-        <v>1</v>
-      </c>
-      <c r="AF4">
-        <v>1</v>
-      </c>
-      <c r="AH4">
-        <v>1</v>
-      </c>
-      <c r="AI4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="Z4">
+        <v>1</v>
+      </c>
+      <c r="AB4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1076,7 +980,7 @@
         <v>91</v>
       </c>
       <c r="Q5" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="R5">
         <v>0</v>
@@ -1088,40 +992,25 @@
         <v>1</v>
       </c>
       <c r="U5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V5">
         <v>2</v>
       </c>
       <c r="X5">
-        <v>2</v>
-      </c>
-      <c r="Y5">
-        <v>1</v>
-      </c>
-      <c r="AA5">
+        <v>3</v>
+      </c>
+      <c r="Z5">
+        <v>3</v>
+      </c>
+      <c r="AB5">
         <v>3</v>
       </c>
       <c r="AC5">
-        <v>3</v>
-      </c>
-      <c r="AD5">
-        <v>2</v>
-      </c>
-      <c r="AF5">
-        <v>3</v>
-      </c>
-      <c r="AG5">
-        <v>1</v>
-      </c>
-      <c r="AH5">
-        <v>3</v>
-      </c>
-      <c r="AI5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1181,7 +1070,7 @@
         <v>70</v>
       </c>
       <c r="Q6" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="R6">
         <v>0</v>
@@ -1193,7 +1082,7 @@
         <v>1</v>
       </c>
       <c r="U6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="V6">
         <v>1</v>
@@ -1202,10 +1091,7 @@
         <v>1</v>
       </c>
       <c r="X6">
-        <v>2</v>
-      </c>
-      <c r="Y6">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="Z6">
         <v>1</v>
@@ -1219,23 +1105,8 @@
       <c r="AC6">
         <v>1</v>
       </c>
-      <c r="AD6">
-        <v>1</v>
-      </c>
-      <c r="AE6">
-        <v>1</v>
-      </c>
-      <c r="AF6">
-        <v>2</v>
-      </c>
-      <c r="AH6">
-        <v>1</v>
-      </c>
-      <c r="AI6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1295,19 +1166,19 @@
         <v>95</v>
       </c>
       <c r="Q7" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="R7">
         <v>2</v>
       </c>
       <c r="S7">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="T7">
         <v>3</v>
       </c>
       <c r="U7">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="V7">
         <v>3</v>
@@ -1316,34 +1187,22 @@
         <v>1</v>
       </c>
       <c r="X7">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="Y7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z7">
-        <v>1</v>
-      </c>
-      <c r="AA7">
-        <v>3</v>
+        <v>3</v>
+      </c>
+      <c r="AB7">
+        <v>4</v>
       </c>
       <c r="AC7">
-        <v>4</v>
-      </c>
-      <c r="AD7">
-        <v>1</v>
-      </c>
-      <c r="AF7">
-        <v>3</v>
-      </c>
-      <c r="AH7">
-        <v>4</v>
-      </c>
-      <c r="AI7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1403,49 +1262,37 @@
         <v>66</v>
       </c>
       <c r="Q8" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="R8">
         <v>2</v>
       </c>
       <c r="S8">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="T8">
         <v>2</v>
       </c>
       <c r="U8">
+        <v>16</v>
+      </c>
+      <c r="V8">
+        <v>2</v>
+      </c>
+      <c r="X8">
+        <v>16</v>
+      </c>
+      <c r="Z8">
+        <v>2</v>
+      </c>
+      <c r="AB8">
         <v>4</v>
       </c>
-      <c r="V8">
-        <v>2</v>
-      </c>
-      <c r="X8">
-        <v>4</v>
-      </c>
-      <c r="Y8">
-        <v>0</v>
-      </c>
-      <c r="AA8">
-        <v>2</v>
-      </c>
       <c r="AC8">
-        <v>4</v>
-      </c>
-      <c r="AD8">
-        <v>1</v>
-      </c>
-      <c r="AF8">
-        <v>2</v>
-      </c>
-      <c r="AH8">
-        <v>4</v>
-      </c>
-      <c r="AI8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1505,52 +1352,37 @@
         <v>90</v>
       </c>
       <c r="Q9" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="R9">
         <v>2</v>
       </c>
       <c r="S9">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="T9">
         <v>2</v>
       </c>
       <c r="U9">
+        <v>17</v>
+      </c>
+      <c r="V9">
+        <v>3</v>
+      </c>
+      <c r="X9">
+        <v>18</v>
+      </c>
+      <c r="Z9">
+        <v>3</v>
+      </c>
+      <c r="AB9">
         <v>4</v>
       </c>
-      <c r="V9">
-        <v>3</v>
-      </c>
-      <c r="X9">
-        <v>5</v>
-      </c>
-      <c r="Y9">
-        <v>1</v>
-      </c>
-      <c r="AA9">
-        <v>3</v>
-      </c>
       <c r="AC9">
-        <v>4</v>
-      </c>
-      <c r="AD9">
-        <v>1</v>
-      </c>
-      <c r="AE9">
-        <v>1</v>
-      </c>
-      <c r="AF9">
-        <v>3</v>
-      </c>
-      <c r="AH9">
-        <v>4</v>
-      </c>
-      <c r="AI9">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1610,45 +1442,33 @@
         <v>80</v>
       </c>
       <c r="Q10" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="R10">
         <v>3</v>
       </c>
       <c r="S10">
+        <v>21</v>
+      </c>
+      <c r="T10">
+        <v>3</v>
+      </c>
+      <c r="U10">
+        <v>21</v>
+      </c>
+      <c r="V10">
+        <v>3</v>
+      </c>
+      <c r="X10">
+        <v>21</v>
+      </c>
+      <c r="Z10">
+        <v>3</v>
+      </c>
+      <c r="AB10">
         <v>5</v>
       </c>
-      <c r="T10">
-        <v>3</v>
-      </c>
-      <c r="U10">
-        <v>5</v>
-      </c>
-      <c r="V10">
-        <v>3</v>
-      </c>
-      <c r="X10">
-        <v>5</v>
-      </c>
-      <c r="Y10">
-        <v>0</v>
-      </c>
-      <c r="AA10">
-        <v>3</v>
-      </c>
       <c r="AC10">
-        <v>5</v>
-      </c>
-      <c r="AD10">
-        <v>0</v>
-      </c>
-      <c r="AF10">
-        <v>3</v>
-      </c>
-      <c r="AH10">
-        <v>5</v>
-      </c>
-      <c r="AI10">
         <v>0</v>
       </c>
     </row>
@@ -1667,7 +1487,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>56</v>
+        <v>37</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -1682,22 +1502,22 @@
         <v>2</v>
       </c>
       <c r="G1" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="H1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="I1" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="J1" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="K1" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="L1" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
@@ -1727,7 +1547,7 @@
         <v>90</v>
       </c>
       <c r="H2" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
@@ -1784,7 +1604,7 @@
         <v>20</v>
       </c>
       <c r="H4" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -1841,7 +1661,7 @@
         <v>90</v>
       </c>
       <c r="H6" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
@@ -1925,7 +1745,7 @@
         <v>100</v>
       </c>
       <c r="H9" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="I9">
         <v>50</v>
@@ -2081,7 +1901,7 @@
         <v>70</v>
       </c>
       <c r="H13" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="I13">
         <v>50</v>
@@ -2249,7 +2069,7 @@
         <v>100</v>
       </c>
       <c r="H18" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="J18">
         <v>65</v>

</xml_diff>

<commit_message>
Fix screening in lesion state
</commit_message>
<xml_diff>
--- a/tests/test_screening_data.xlsx
+++ b/tests/test_screening_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85CEEFDA-E9C5-C84D-9121-81193C7A5F92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE50839D-CBD9-9F44-BEA4-2CE63DCA8ABC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" activeTab="1" xr2:uid="{C01DA78E-62CC-6E49-850F-A2DB27289041}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17760" xr2:uid="{C01DA78E-62CC-6E49-850F-A2DB27289041}"/>
   </bookViews>
   <sheets>
     <sheet name="m_patient" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="48">
   <si>
     <t>pt_id</t>
   </si>
@@ -141,15 +141,6 @@
     <t>preclinical detection</t>
   </si>
   <si>
-    <t>test_2_nosurv_time_detected</t>
-  </si>
-  <si>
-    <t>test_1_surv_time_detected</t>
-  </si>
-  <si>
-    <t>test_2_surv_time_detected</t>
-  </si>
-  <si>
     <t>lesion_id</t>
   </si>
   <si>
@@ -187,6 +178,9 @@
   </si>
   <si>
     <t>test_10_time_detected</t>
+  </si>
+  <si>
+    <t>test_1_time_detected</t>
   </si>
 </sst>
 </file>
@@ -614,40 +608,40 @@
         <v>19</v>
       </c>
       <c r="R1" t="s">
+        <v>35</v>
+      </c>
+      <c r="S1" t="s">
+        <v>36</v>
+      </c>
+      <c r="T1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U1" t="s">
         <v>38</v>
       </c>
-      <c r="S1" t="s">
+      <c r="V1" t="s">
         <v>39</v>
       </c>
-      <c r="T1" t="s">
+      <c r="W1" t="s">
         <v>40</v>
       </c>
-      <c r="U1" t="s">
+      <c r="X1" t="s">
         <v>41</v>
-      </c>
-      <c r="V1" t="s">
-        <v>42</v>
-      </c>
-      <c r="W1" t="s">
-        <v>43</v>
-      </c>
-      <c r="X1" t="s">
-        <v>44</v>
       </c>
       <c r="Y1" t="s">
         <v>7</v>
       </c>
       <c r="Z1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="AA1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="AB1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="AC1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:29" x14ac:dyDescent="0.2">
@@ -745,6 +739,9 @@
       <c r="AB2">
         <v>0</v>
       </c>
+      <c r="AC2">
+        <v>1</v>
+      </c>
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A3">
@@ -1004,10 +1001,7 @@
         <v>3</v>
       </c>
       <c r="AB5">
-        <v>3</v>
-      </c>
-      <c r="AC5">
-        <v>2</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.2">
@@ -1100,10 +1094,7 @@
         <v>1</v>
       </c>
       <c r="AB6">
-        <v>1</v>
-      </c>
-      <c r="AC6">
-        <v>1</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.2">
@@ -1196,10 +1187,7 @@
         <v>3</v>
       </c>
       <c r="AB7">
-        <v>4</v>
-      </c>
-      <c r="AC7">
-        <v>1</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.2">
@@ -1286,10 +1274,7 @@
         <v>2</v>
       </c>
       <c r="AB8">
-        <v>4</v>
-      </c>
-      <c r="AC8">
-        <v>1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.2">
@@ -1376,10 +1361,7 @@
         <v>3</v>
       </c>
       <c r="AB9">
-        <v>4</v>
-      </c>
-      <c r="AC9">
-        <v>1</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2">
@@ -1466,10 +1448,7 @@
         <v>3</v>
       </c>
       <c r="AB10">
-        <v>5</v>
-      </c>
-      <c r="AC10">
-        <v>0</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1479,15 +1458,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFC853AB-1B40-724B-B920-12502C063EDC}">
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -1508,19 +1487,13 @@
         <v>19</v>
       </c>
       <c r="I1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="J1" t="s">
-        <v>34</v>
-      </c>
-      <c r="K1" t="s">
-        <v>35</v>
-      </c>
-      <c r="L1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1550,7 +1523,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1577,7 +1550,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1607,7 +1580,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2</v>
       </c>
@@ -1634,7 +1607,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>3</v>
       </c>
@@ -1664,7 +1637,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>3</v>
       </c>
@@ -1691,7 +1664,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>3</v>
       </c>
@@ -1718,7 +1691,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>4</v>
       </c>
@@ -1753,14 +1726,8 @@
       <c r="J9">
         <v>50</v>
       </c>
-      <c r="K9">
-        <v>50</v>
-      </c>
-      <c r="L9">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>4</v>
       </c>
@@ -1792,14 +1759,8 @@
       <c r="J10">
         <v>50</v>
       </c>
-      <c r="K10">
-        <v>50</v>
-      </c>
-      <c r="L10">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>4</v>
       </c>
@@ -1831,14 +1792,8 @@
       <c r="J11">
         <v>50</v>
       </c>
-      <c r="K11">
-        <v>50</v>
-      </c>
-      <c r="L11">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>4</v>
       </c>
@@ -1870,11 +1825,8 @@
       <c r="J12">
         <v>65</v>
       </c>
-      <c r="L12">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>5</v>
       </c>
@@ -1909,14 +1861,8 @@
       <c r="J13">
         <v>50</v>
       </c>
-      <c r="K13">
-        <v>50</v>
-      </c>
-      <c r="L13">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>5</v>
       </c>
@@ -1942,8 +1888,11 @@
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A14,m_patient!$A:$A,0))</f>
         <v>70</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="J14">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>5</v>
       </c>
@@ -1969,8 +1918,11 @@
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A15,m_patient!$A:$A,0))</f>
         <v>70</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="J15">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>6</v>
       </c>
@@ -2000,16 +1952,10 @@
         <v>70</v>
       </c>
       <c r="J16">
-        <v>65</v>
-      </c>
-      <c r="K16">
-        <v>70</v>
-      </c>
-      <c r="L16">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>7</v>
       </c>
@@ -2036,13 +1982,10 @@
         <v>66</v>
       </c>
       <c r="J17">
-        <v>65</v>
-      </c>
-      <c r="L17">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>8</v>
       </c>
@@ -2072,13 +2015,10 @@
         <v>31</v>
       </c>
       <c r="J18">
-        <v>65</v>
-      </c>
-      <c r="L18">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>8</v>
       </c>
@@ -2105,13 +2045,10 @@
         <v>100</v>
       </c>
       <c r="J19">
-        <v>65</v>
-      </c>
-      <c r="L19">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>8</v>
       </c>
@@ -2138,13 +2075,10 @@
         <v>100</v>
       </c>
       <c r="J20">
-        <v>65</v>
-      </c>
-      <c r="L20">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>8</v>
       </c>
@@ -2171,13 +2105,10 @@
         <v>100</v>
       </c>
       <c r="J21">
-        <v>65</v>
-      </c>
-      <c r="L21">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>8</v>
       </c>
@@ -2202,11 +2133,11 @@
         <f>INDEX(m_patient!O:O,MATCH(m_lesion!$A22,m_patient!$A:$A,0))</f>
         <v>100</v>
       </c>
-      <c r="L22">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="J22">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
Add unit tests for multiple screening tests, clean folders
</commit_message>
<xml_diff>
--- a/tests/test_screening_data.xlsx
+++ b/tests/test_screening_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE50839D-CBD9-9F44-BEA4-2CE63DCA8ABC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E27C305B-21E8-1D44-9D66-0B08C4FAF595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17760" xr2:uid="{C01DA78E-62CC-6E49-850F-A2DB27289041}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="52">
   <si>
     <t>pt_id</t>
   </si>
@@ -181,6 +181,18 @@
   </si>
   <si>
     <t>test_1_time_detected</t>
+  </si>
+  <si>
+    <t>ct_10_pos_P</t>
+  </si>
+  <si>
+    <t>ct_1_pos_P</t>
+  </si>
+  <si>
+    <t>ct_10_pos_L</t>
+  </si>
+  <si>
+    <t>ct_1_pos_L</t>
   </si>
 </sst>
 </file>
@@ -552,10 +564,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE386AE5-7C58-FF46-B22F-83A12B65CF2D}">
-  <dimension ref="A1:AC10"/>
+  <dimension ref="A1:AG10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -626,25 +638,37 @@
         <v>40</v>
       </c>
       <c r="X1" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y1" t="s">
         <v>41</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>7</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AB1" t="s">
         <v>44</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AC1" t="s">
         <v>45</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AD1" t="s">
+        <v>50</v>
+      </c>
+      <c r="AE1" t="s">
         <v>42</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AF1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="AG1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -728,13 +752,13 @@
         <v>0</v>
       </c>
       <c r="Y2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB2">
         <v>0</v>
@@ -742,8 +766,20 @@
       <c r="AC2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="AD2">
+        <v>0</v>
+      </c>
+      <c r="AE2">
+        <v>0</v>
+      </c>
+      <c r="AF2">
+        <v>1</v>
+      </c>
+      <c r="AG2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -823,14 +859,26 @@
       <c r="X3">
         <v>0</v>
       </c>
-      <c r="Z3">
+      <c r="Y3">
+        <v>0</v>
+      </c>
+      <c r="AA3">
         <v>0</v>
       </c>
       <c r="AB3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="AD3">
+        <v>0</v>
+      </c>
+      <c r="AE3">
+        <v>0</v>
+      </c>
+      <c r="AG3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -910,14 +958,26 @@
       <c r="X4">
         <v>1</v>
       </c>
-      <c r="Z4">
+      <c r="Y4">
+        <v>1</v>
+      </c>
+      <c r="AA4">
         <v>1</v>
       </c>
       <c r="AB4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="AD4">
+        <v>1</v>
+      </c>
+      <c r="AE4">
+        <v>1</v>
+      </c>
+      <c r="AG4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -995,16 +1055,28 @@
         <v>2</v>
       </c>
       <c r="X5">
-        <v>3</v>
-      </c>
-      <c r="Z5">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="Y5">
+        <v>3</v>
+      </c>
+      <c r="AA5">
+        <v>1</v>
       </c>
       <c r="AB5">
+        <v>3</v>
+      </c>
+      <c r="AD5">
+        <v>2</v>
+      </c>
+      <c r="AE5">
         <v>21</v>
       </c>
-    </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="AG5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1085,19 +1157,31 @@
         <v>1</v>
       </c>
       <c r="X6">
+        <v>0</v>
+      </c>
+      <c r="Y6">
         <v>7</v>
       </c>
-      <c r="Z6">
-        <v>1</v>
-      </c>
       <c r="AA6">
         <v>1</v>
       </c>
       <c r="AB6">
+        <v>1</v>
+      </c>
+      <c r="AC6">
+        <v>1</v>
+      </c>
+      <c r="AD6">
+        <v>1</v>
+      </c>
+      <c r="AE6">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="AG6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1178,19 +1262,31 @@
         <v>1</v>
       </c>
       <c r="X7">
+        <v>0</v>
+      </c>
+      <c r="Y7">
         <v>21</v>
       </c>
-      <c r="Y7">
-        <v>1</v>
-      </c>
       <c r="Z7">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="AA7">
+        <v>0</v>
       </c>
       <c r="AB7">
+        <v>3</v>
+      </c>
+      <c r="AD7">
+        <v>1</v>
+      </c>
+      <c r="AE7">
         <v>21</v>
       </c>
-    </row>
-    <row r="8" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="AG7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1268,16 +1364,28 @@
         <v>2</v>
       </c>
       <c r="X8">
+        <v>0</v>
+      </c>
+      <c r="Y8">
         <v>16</v>
       </c>
-      <c r="Z8">
-        <v>2</v>
+      <c r="AA8">
+        <v>0</v>
       </c>
       <c r="AB8">
+        <v>2</v>
+      </c>
+      <c r="AD8">
+        <v>0</v>
+      </c>
+      <c r="AE8">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="AG8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1355,16 +1463,28 @@
         <v>3</v>
       </c>
       <c r="X9">
+        <v>1</v>
+      </c>
+      <c r="Y9">
         <v>18</v>
       </c>
-      <c r="Z9">
-        <v>3</v>
+      <c r="AA9">
+        <v>1</v>
       </c>
       <c r="AB9">
+        <v>3</v>
+      </c>
+      <c r="AD9">
+        <v>1</v>
+      </c>
+      <c r="AE9">
         <v>21</v>
       </c>
-    </row>
-    <row r="10" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="AG9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1442,13 +1562,25 @@
         <v>3</v>
       </c>
       <c r="X10">
+        <v>0</v>
+      </c>
+      <c r="Y10">
         <v>21</v>
       </c>
-      <c r="Z10">
-        <v>3</v>
+      <c r="AA10">
+        <v>0</v>
       </c>
       <c r="AB10">
+        <v>3</v>
+      </c>
+      <c r="AD10">
+        <v>0</v>
+      </c>
+      <c r="AE10">
         <v>21</v>
+      </c>
+      <c r="AG10">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>